<commit_message>
Mountain Trade payroll items priced at staff rate (moving to Jessica)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRgGtk6aohavQBQTYDwapz
</commit_message>
<xml_diff>
--- a/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
+++ b/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
@@ -4758,7 +4758,7 @@
       </c>
       <c r="E69" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F75*IF(H69="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="F69" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G75*60,0)/1440</f>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="H69" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L75</f>
-        <v>CFO</v>
+        <v>Staff</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="E70" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F76*IF(H70="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>229</v>
+        <v>87</v>
       </c>
       <c r="F70" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G76*60,0)/1440</f>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="H70" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L76</f>
-        <v>CFO</v>
+        <v>Staff</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15109,11 +15109,11 @@
         <v>0</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>185</v>
+        <v>87</v>
       </c>
       <c r="M75" s="22" t="n">
         <f aca="false">F75*IF(L75="CFO",Assumptions!$B$5,Assumptions!$B$4)+G75*Assumptions!$B$5</f>
-        <v>83.325</v>
+        <v>31.6635</v>
       </c>
       <c r="N75" s="16" t="n">
         <f aca="false">F75*INDEX(Assumptions!$B$8:$B$14,MATCH(E75,Assumptions!$A$8:$A$14,0))</f>
@@ -15172,11 +15172,11 @@
         <v>15</v>
       </c>
       <c r="L76" s="9" t="s">
-        <v>185</v>
+        <v>87</v>
       </c>
       <c r="M76" s="22" t="n">
         <f aca="false">F76*IF(L76="CFO",Assumptions!$B$5,Assumptions!$B$4)+G76*Assumptions!$B$5</f>
-        <v>291.675</v>
+        <v>149.5865</v>
       </c>
       <c r="N76" s="16" t="n">
         <f aca="false">F76*INDEX(Assumptions!$B$8:$B$14,MATCH(E76,Assumptions!$A$8:$A$14,0))</f>
@@ -23829,7 +23829,7 @@
       </c>
       <c r="M105" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P105,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>291.675</v>
+        <v>149.5865</v>
       </c>
       <c r="N105" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P105,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -23886,7 +23886,7 @@
       </c>
       <c r="M106" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P106,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>83.325</v>
+        <v>31.6635</v>
       </c>
       <c r="N106" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P106,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -28270,7 +28270,7 @@
       </c>
       <c r="M186" s="32" t="n">
         <f aca="false">SUM(M2:M184)</f>
-        <v>72508.356</v>
+        <v>72314.606</v>
       </c>
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>

</xml_diff>

<commit_message>
Apply Josephine's 1099 tier edits to the master workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRgGtk6aohavQBQTYDwapz
</commit_message>
<xml_diff>
--- a/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
+++ b/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
@@ -800,6 +800,9 @@
     <t xml:space="preserve">7327 Tierra Buena LLC|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
+    <t xml:space="preserve">1099 tier Standard: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle.</t>
+  </si>
+  <si>
     <t xml:space="preserve">7327 Tierra Buena LLC|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
@@ -842,36 +845,36 @@
     <t xml:space="preserve">Amerisource HR Consulting Group LLC|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
+    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Year-end review|Adjusting Journal Entry Request|Annual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year-end review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year-end/tax hours Oct 2025–Sep 2026 (5.6h).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Monthly Financials|Month End Close|Monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Includes Month-end 5.0, Payroll 11.7, CFO advisory 0.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Bookkeeping|Bookkeeping &amp; Bill Pay|Weekly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bookkeeping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly bookkeeping/settlement time ÷ weeks per month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSD Contracting LLC|1099|1099 Quarterly Review|1099</t>
+  </si>
+  <si>
     <t xml:space="preserve">1099 tier Complex: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle.</t>
   </si>
   <si>
-    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Year-end review|Adjusting Journal Entry Request|Annual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year-end review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year-end/tax hours Oct 2025–Sep 2026 (5.6h).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Monthly Financials|Month End Close|Monthly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Includes Month-end 5.0, Payroll 11.7, CFO advisory 0.2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amerisource HR Consulting Group LLC|Bookkeeping|Bookkeeping &amp; Bill Pay|Weekly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bookkeeping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly bookkeeping/settlement time ÷ weeks per month.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSD Contracting LLC|1099|1099 Quarterly Review|1099</t>
-  </si>
-  <si>
     <t xml:space="preserve">BSD Contracting LLC|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
@@ -896,9 +899,6 @@
     <t xml:space="preserve">BeckShar Development LLC|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
-    <t xml:space="preserve">1099 tier Standard: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle.</t>
-  </si>
-  <si>
     <t xml:space="preserve">BeckShar Development LLC|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
@@ -935,7 +935,7 @@
     <t xml:space="preserve">Capital Financial LLC|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
-    <t xml:space="preserve">1099 tier Complex: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Aug–Sep 2026 excluded (one-time payroll JE re-entry, resolved).</t>
+    <t xml:space="preserve">1099 tier Standard: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Aug–Sep 2026 excluded (one-time payroll JE re-entry, resolved).</t>
   </si>
   <si>
     <t xml:space="preserve">Settled from 2026-03 (2026-03 – 2026-07)</t>
@@ -1304,7 +1304,7 @@
     <t xml:space="preserve">Southwest Rents Inc|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
-    <t xml:space="preserve">1099 tier Standard: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h).</t>
+    <t xml:space="preserve">1099 tier Complex: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h).</t>
   </si>
   <si>
     <t xml:space="preserve">Southwest Rents Inc|Year-end review|Adjusting Journal Entry Request|Annual</t>
@@ -1322,7 +1322,7 @@
     <t xml:space="preserve">T5 Family Holdings LLC|1099|1099 Quarterly Review|1099</t>
   </si>
   <si>
-    <t xml:space="preserve">1099 tier Standard: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Carries Tavasci Group shared work since Harvest (moved from ESH). Group weekly items under Phil Tavasci Companies are budgeted from T5 history.</t>
+    <t xml:space="preserve">1099 tier Simple: ongoing quarterly review (half a full review). See 1099 tab for the Oct 30 cycle. Carries Tavasci Group shared work since Harvest (moved from ESH). Group weekly items under Phil Tavasci Companies are budgeted from T5 history.</t>
   </si>
   <si>
     <t xml:space="preserve">T5 Family Holdings LLC|Monthly Financials|Month End Close|Monthly</t>
@@ -3111,11 +3111,11 @@
       </c>
       <c r="D16" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F12*60,0)/1440</f>
-        <v>0.0520833333333333</v>
+        <v>0.03125</v>
       </c>
       <c r="E16" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F12*IF(H16="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>119</v>
+        <v>71</v>
       </c>
       <c r="F16" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G12*60,0)/1440</f>
@@ -3297,11 +3297,11 @@
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F18*60,0)/1440</f>
-        <v>0.0833333333333333</v>
+        <v>0.03125</v>
       </c>
       <c r="E22" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F18*IF(H22="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>190</v>
+        <v>71</v>
       </c>
       <c r="F22" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G18*60,0)/1440</f>
@@ -3731,11 +3731,11 @@
       </c>
       <c r="D36" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F32*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="E36" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F32*IF(H36="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>190</v>
       </c>
       <c r="F36" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G32*60,0)/1440</f>
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D38" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F34*60,0)/1440</f>
-        <v>0.0833333333333333</v>
+        <v>0.03125</v>
       </c>
       <c r="E38" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F34*IF(H38="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>190</v>
+        <v>71</v>
       </c>
       <c r="F38" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G34*60,0)/1440</f>
@@ -4196,11 +4196,11 @@
       </c>
       <c r="D51" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F48*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="E51" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F48*IF(H51="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>190</v>
       </c>
       <c r="F51" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G48*60,0)/1440</f>
@@ -4351,11 +4351,11 @@
       </c>
       <c r="D56" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F62*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0159722222222222</v>
       </c>
       <c r="E56" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F62*IF(H56="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="F56" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G62*60,0)/1440</f>
@@ -5622,11 +5622,11 @@
       </c>
       <c r="D97" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F103*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="E97" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F103*IF(H97="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>190</v>
       </c>
       <c r="F97" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G103*60,0)/1440</f>
@@ -5715,11 +5715,11 @@
       </c>
       <c r="D100" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F106*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0159722222222222</v>
       </c>
       <c r="E100" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F106*IF(H100="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="F100" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G106*60,0)/1440</f>
@@ -6503,11 +6503,11 @@
       </c>
       <c r="D127" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I15*60,0)/1440</f>
-        <v>0.104166666666667</v>
+        <v>0.0625</v>
       </c>
       <c r="E127" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I15*IF(H127="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>238</v>
+        <v>143</v>
       </c>
       <c r="F127" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J15*60,0)/1440</f>
@@ -6593,11 +6593,11 @@
       </c>
       <c r="D130" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I23*60,0)/1440</f>
-        <v>0.0833333333333333</v>
+        <v>0.03125</v>
       </c>
       <c r="E130" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I23*IF(H130="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>190</v>
+        <v>71</v>
       </c>
       <c r="F130" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J23*60,0)/1440</f>
@@ -6863,11 +6863,11 @@
       </c>
       <c r="D139" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I44*60,0)/1440</f>
-        <v>0.0625</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="E139" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I44*IF(H139="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>143</v>
+        <v>380</v>
       </c>
       <c r="F139" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J44*60,0)/1440</f>
@@ -6923,11 +6923,11 @@
       </c>
       <c r="D141" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I47*60,0)/1440</f>
-        <v>0.0833333333333333</v>
+        <v>0.03125</v>
       </c>
       <c r="E141" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I47*IF(H141="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>190</v>
+        <v>71</v>
       </c>
       <c r="F141" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J47*60,0)/1440</f>
@@ -7163,11 +7163,11 @@
       </c>
       <c r="D149" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I66*60,0)/1440</f>
-        <v>0.0625</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="E149" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I66*IF(H149="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>143</v>
+        <v>380</v>
       </c>
       <c r="F149" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J66*60,0)/1440</f>
@@ -7223,11 +7223,11 @@
       </c>
       <c r="D151" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I88*60,0)/1440</f>
-        <v>0.03125</v>
+        <v>0.0159722222222222</v>
       </c>
       <c r="E151" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I88*IF(H151="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="F151" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J88*60,0)/1440</f>
@@ -8033,11 +8033,11 @@
       </c>
       <c r="D178" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I157*60,0)/1440</f>
-        <v>0.0625</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="E178" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I157*IF(H178="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>143</v>
+        <v>380</v>
       </c>
       <c r="F178" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J157*60,0)/1440</f>
@@ -8063,11 +8063,11 @@
       </c>
       <c r="D179" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I160*60,0)/1440</f>
-        <v>0.0472222222222222</v>
+        <v>0.0236111111111111</v>
       </c>
       <c r="E179" s="7" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!I160*IF(H179="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>107</v>
+        <v>53</v>
       </c>
       <c r="F179" s="6" t="n">
         <f aca="false">ROUND('Open Items (Karbon)'!J160*60,0)/1440</f>
@@ -9273,14 +9273,14 @@
         <v>24</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>177</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B9,Assumptions!$A$17:$A$20,0))</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E9" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C9,Assumptions!$A$23:$A$27,0))</f>
@@ -9288,15 +9288,15 @@
       </c>
       <c r="F9" s="17" t="n">
         <f aca="false">D9*E9</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">ROUND(F9*60,0)</f>
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="H9" s="16" t="n">
         <f aca="false">IF(C9="Excluded (in-house)",0,D9*Assumptions!$B$29)</f>
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="I9" s="15" t="n">
         <v>0</v>
@@ -9378,14 +9378,14 @@
         <v>27</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>173</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B12,Assumptions!$A$17:$A$20,0))</f>
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="E12" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C12,Assumptions!$A$23:$A$27,0))</f>
@@ -9393,15 +9393,15 @@
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">D12*E12</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="G12" s="10" t="n">
         <f aca="false">ROUND(F12*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="H12" s="16" t="n">
         <f aca="false">IF(C12="Excluded (in-house)",0,D12*Assumptions!$B$29)</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="I12" s="15" t="n">
         <v>4.5</v>
@@ -9555,14 +9555,14 @@
         <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>177</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B17,Assumptions!$A$17:$A$20,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="E17" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C17,Assumptions!$A$23:$A$27,0))</f>
@@ -9570,15 +9570,15 @@
       </c>
       <c r="F17" s="17" t="n">
         <f aca="false">D17*E17</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="G17" s="10" t="n">
         <f aca="false">ROUND(F17*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="H17" s="16" t="n">
         <f aca="false">IF(C17="Excluded (in-house)",0,D17*Assumptions!$B$29)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I17" s="15" t="n">
         <v>0</v>
@@ -9590,14 +9590,14 @@
         <v>37</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>173</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B18,Assumptions!$A$17:$A$20,0))</f>
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="E18" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C18,Assumptions!$A$23:$A$27,0))</f>
@@ -9605,15 +9605,15 @@
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">D18*E18</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="G18" s="10" t="n">
         <f aca="false">ROUND(F18*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="H18" s="16" t="n">
         <f aca="false">IF(C18="Excluded (in-house)",0,D18*Assumptions!$B$29)</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="I18" s="15" t="n">
         <v>3</v>
@@ -9769,14 +9769,14 @@
         <v>45</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>177</v>
       </c>
       <c r="D23" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B23,Assumptions!$A$17:$A$20,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="E23" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C23,Assumptions!$A$23:$A$27,0))</f>
@@ -9784,15 +9784,15 @@
       </c>
       <c r="F23" s="17" t="n">
         <f aca="false">D23*E23</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="G23" s="10" t="n">
         <f aca="false">ROUND(F23*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="H23" s="16" t="n">
         <f aca="false">IF(C23="Excluded (in-house)",0,D23*Assumptions!$B$29)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I23" s="15" t="n">
         <v>0</v>
@@ -9878,14 +9878,14 @@
         <v>47</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>173</v>
       </c>
       <c r="D26" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B26,Assumptions!$A$17:$A$20,0))</f>
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="E26" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C26,Assumptions!$A$23:$A$27,0))</f>
@@ -9893,15 +9893,15 @@
       </c>
       <c r="F26" s="17" t="n">
         <f aca="false">D26*E26</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="G26" s="10" t="n">
         <f aca="false">ROUND(F26*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="H26" s="16" t="n">
         <f aca="false">IF(C26="Excluded (in-house)",0,D26*Assumptions!$B$29)</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="I26" s="15" t="n">
         <v>1</v>
@@ -10341,14 +10341,14 @@
         <v>73</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>177</v>
       </c>
       <c r="D39" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B39,Assumptions!$A$17:$A$20,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C39,Assumptions!$A$23:$A$27,0))</f>
@@ -10356,15 +10356,15 @@
       </c>
       <c r="F39" s="17" t="n">
         <f aca="false">D39*E39</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="G39" s="10" t="n">
         <f aca="false">ROUND(F39*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="H39" s="16" t="n">
         <f aca="false">IF(C39="Excluded (in-house)",0,D39*Assumptions!$B$29)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I39" s="15" t="n">
         <v>0</v>
@@ -10376,14 +10376,14 @@
         <v>74</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>175</v>
       </c>
       <c r="D40" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$17:$B$20,MATCH(B40,Assumptions!$A$17:$A$20,0))</f>
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="E40" s="16" t="n">
         <f aca="false">INDEX(Assumptions!$B$23:$B$27,MATCH(C40,Assumptions!$A$23:$A$27,0))</f>
@@ -10391,15 +10391,15 @@
       </c>
       <c r="F40" s="17" t="n">
         <f aca="false">D40*E40</f>
-        <v>1.125</v>
+        <v>0.5625</v>
       </c>
       <c r="G40" s="10" t="n">
         <f aca="false">ROUND(F40*60,0)</f>
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="H40" s="16" t="n">
         <f aca="false">IF(C40="Excluded (in-house)",0,D40*Assumptions!$B$29)</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="I40" s="15" t="n">
         <v>0.75</v>
@@ -10591,11 +10591,11 @@
       <c r="E46" s="2"/>
       <c r="F46" s="19" t="n">
         <f aca="false">SUM(F5:F45)</f>
-        <v>71.75</v>
+        <v>74.8125</v>
       </c>
       <c r="G46" s="20" t="n">
         <f aca="false">SUM(G5:G45)</f>
-        <v>4309</v>
+        <v>4493</v>
       </c>
       <c r="H46" s="19" t="n">
         <f aca="false">SUM(H5:H45)</f>
@@ -11387,22 +11387,22 @@
       </c>
       <c r="F12" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B12,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="21" t="n">
         <f aca="false">F12+G12</f>
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="I12" s="2" t="n">
         <f aca="false">ROUND(H12*60,0)</f>
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J12" s="2" t="n">
         <f aca="false">ROUND(F12*60,0)</f>
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="K12" s="2" t="n">
         <f aca="false">ROUND(G12*60,0)</f>
@@ -11413,11 +11413,11 @@
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">F12*IF(L12="CFO",Assumptions!$B$5,Assumptions!$B$4)+G12*Assumptions!$B$5</f>
-        <v>118.75</v>
+        <v>71.25</v>
       </c>
       <c r="N12" s="16" t="n">
         <f aca="false">F12*INDEX(Assumptions!$B$8:$B$14,MATCH(E12,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.416666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="O12" s="16" t="n">
         <f aca="false">G12*INDEX(Assumptions!$B$8:$B$14,MATCH(E12,Assumptions!$A$8:$A$14,0))</f>
@@ -11427,7 +11427,7 @@
         <v>227</v>
       </c>
       <c r="Q12" s="24" t="s">
-        <v>228</v>
+        <v>255</v>
       </c>
       <c r="R12" s="2" t="s">
         <v>251</v>
@@ -11435,7 +11435,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>24</v>
@@ -11490,7 +11490,7 @@
         <v>232</v>
       </c>
       <c r="Q13" s="24" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="R13" s="2" t="s">
         <v>251</v>
@@ -11498,7 +11498,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>25</v>
@@ -11554,15 +11554,15 @@
         <v>227</v>
       </c>
       <c r="Q14" s="24" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>25</v>
@@ -11614,18 +11614,18 @@
         <v>0.25</v>
       </c>
       <c r="P15" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q15" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>26</v>
@@ -11678,10 +11678,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q16" s="24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R16" s="2" t="s">
         <v>229</v>
@@ -11689,7 +11689,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>26</v>
@@ -11741,10 +11741,10 @@
         <v>0.3333</v>
       </c>
       <c r="P17" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q17" s="24" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R17" s="2" t="s">
         <v>229</v>
@@ -11752,7 +11752,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>27</v>
@@ -11768,22 +11768,22 @@
       </c>
       <c r="F18" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B18,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="21" t="n">
         <f aca="false">F18+G18</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="I18" s="2" t="n">
         <f aca="false">ROUND(H18*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="J18" s="2" t="n">
         <f aca="false">ROUND(F18*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="K18" s="2" t="n">
         <f aca="false">ROUND(G18*60,0)</f>
@@ -11794,11 +11794,11 @@
       </c>
       <c r="M18" s="22" t="n">
         <f aca="false">F18*IF(L18="CFO",Assumptions!$B$5,Assumptions!$B$4)+G18*Assumptions!$B$5</f>
-        <v>190</v>
+        <v>71.25</v>
       </c>
       <c r="N18" s="16" t="n">
         <f aca="false">F18*INDEX(Assumptions!$B$8:$B$14,MATCH(E18,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="O18" s="16" t="n">
         <f aca="false">G18*INDEX(Assumptions!$B$8:$B$14,MATCH(E18,Assumptions!$A$8:$A$14,0))</f>
@@ -11808,7 +11808,7 @@
         <v>227</v>
       </c>
       <c r="Q18" s="24" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="R18" s="2" t="s">
         <v>247</v>
@@ -12061,15 +12061,15 @@
         <v>227</v>
       </c>
       <c r="Q22" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>31</v>
@@ -12124,15 +12124,15 @@
         <v>232</v>
       </c>
       <c r="Q23" s="24" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R23" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>32</v>
@@ -12187,15 +12187,15 @@
         <v>232</v>
       </c>
       <c r="Q24" s="24" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R24" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>32</v>
@@ -12250,15 +12250,15 @@
         <v>232</v>
       </c>
       <c r="Q25" s="24" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>33</v>
@@ -12314,7 +12314,7 @@
         <v>227</v>
       </c>
       <c r="Q26" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R26" s="2" t="s">
         <v>229</v>
@@ -12441,7 +12441,7 @@
         <v>227</v>
       </c>
       <c r="Q28" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R28" s="2" t="s">
         <v>229</v>
@@ -12568,7 +12568,7 @@
         <v>227</v>
       </c>
       <c r="Q30" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R30" s="2" t="s">
         <v>293</v>
@@ -12655,22 +12655,22 @@
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B32,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="G32" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H32" s="21" t="n">
         <f aca="false">F32+G32</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I32" s="2" t="n">
         <f aca="false">ROUND(H32*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J32" s="2" t="n">
         <f aca="false">ROUND(F32*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="K32" s="2" t="n">
         <f aca="false">ROUND(G32*60,0)</f>
@@ -12681,11 +12681,11 @@
       </c>
       <c r="M32" s="22" t="n">
         <f aca="false">F32*IF(L32="CFO",Assumptions!$B$5,Assumptions!$B$4)+G32*Assumptions!$B$5</f>
-        <v>71.25</v>
+        <v>190</v>
       </c>
       <c r="N32" s="16" t="n">
         <f aca="false">F32*INDEX(Assumptions!$B$8:$B$14,MATCH(E32,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="O32" s="16" t="n">
         <f aca="false">G32*INDEX(Assumptions!$B$8:$B$14,MATCH(E32,Assumptions!$A$8:$A$14,0))</f>
@@ -12695,10 +12695,10 @@
         <v>227</v>
       </c>
       <c r="Q32" s="24" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="R32" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12761,7 +12761,7 @@
         <v>298</v>
       </c>
       <c r="R33" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12782,22 +12782,22 @@
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B34,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="G34" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="21" t="n">
         <f aca="false">F34+G34</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="I34" s="2" t="n">
         <f aca="false">ROUND(H34*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="J34" s="2" t="n">
         <f aca="false">ROUND(F34*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="K34" s="2" t="n">
         <f aca="false">ROUND(G34*60,0)</f>
@@ -12808,11 +12808,11 @@
       </c>
       <c r="M34" s="22" t="n">
         <f aca="false">F34*IF(L34="CFO",Assumptions!$B$5,Assumptions!$B$4)+G34*Assumptions!$B$5</f>
-        <v>190</v>
+        <v>71.25</v>
       </c>
       <c r="N34" s="16" t="n">
         <f aca="false">F34*INDEX(Assumptions!$B$8:$B$14,MATCH(E34,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.666666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="O34" s="16" t="n">
         <f aca="false">G34*INDEX(Assumptions!$B$8:$B$14,MATCH(E34,Assumptions!$A$8:$A$14,0))</f>
@@ -12949,10 +12949,10 @@
         <v>227</v>
       </c>
       <c r="Q36" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R36" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13015,7 +13015,7 @@
         <v>306</v>
       </c>
       <c r="R37" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13076,10 +13076,10 @@
         <v>227</v>
       </c>
       <c r="Q38" s="24" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R38" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13136,13 +13136,13 @@
         <v>0.3333</v>
       </c>
       <c r="P39" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q39" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R39" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13203,7 +13203,7 @@
         <v>227</v>
       </c>
       <c r="Q40" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R40" s="2" t="s">
         <v>310</v>
@@ -13360,7 +13360,7 @@
         <v>0</v>
       </c>
       <c r="P43" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q43" s="24" t="s">
         <v>319</v>
@@ -13429,7 +13429,7 @@
         <v>322</v>
       </c>
       <c r="R44" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13640,22 +13640,22 @@
       </c>
       <c r="F48" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B48,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="G48" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="21" t="n">
         <f aca="false">F48+G48</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I48" s="2" t="n">
         <f aca="false">ROUND(H48*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J48" s="2" t="n">
         <f aca="false">ROUND(F48*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="K48" s="2" t="n">
         <f aca="false">ROUND(G48*60,0)</f>
@@ -13666,11 +13666,11 @@
       </c>
       <c r="M48" s="22" t="n">
         <f aca="false">F48*IF(L48="CFO",Assumptions!$B$5,Assumptions!$B$4)+G48*Assumptions!$B$5</f>
-        <v>71.25</v>
+        <v>190</v>
       </c>
       <c r="N48" s="16" t="n">
         <f aca="false">F48*INDEX(Assumptions!$B$8:$B$14,MATCH(E48,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="O48" s="16" t="n">
         <f aca="false">G48*INDEX(Assumptions!$B$8:$B$14,MATCH(E48,Assumptions!$A$8:$A$14,0))</f>
@@ -13680,7 +13680,7 @@
         <v>227</v>
       </c>
       <c r="Q48" s="24" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="R48" s="2" t="s">
         <v>293</v>
@@ -13744,7 +13744,7 @@
         <v>227</v>
       </c>
       <c r="Q49" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R49" s="2" t="s">
         <v>235</v>
@@ -14263,22 +14263,22 @@
       </c>
       <c r="F62" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B62,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="G62" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="21" t="n">
         <f aca="false">F62+G62</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="I62" s="2" t="n">
         <f aca="false">ROUND(H62*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="J62" s="2" t="n">
         <f aca="false">ROUND(F62*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="K62" s="2" t="n">
         <f aca="false">ROUND(G62*60,0)</f>
@@ -14289,11 +14289,11 @@
       </c>
       <c r="M62" s="22" t="n">
         <f aca="false">F62*IF(L62="CFO",Assumptions!$B$5,Assumptions!$B$4)+G62*Assumptions!$B$5</f>
-        <v>71.25</v>
+        <v>35.625</v>
       </c>
       <c r="N62" s="16" t="n">
         <f aca="false">F62*INDEX(Assumptions!$B$8:$B$14,MATCH(E62,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="O62" s="16" t="n">
         <f aca="false">G62*INDEX(Assumptions!$B$8:$B$14,MATCH(E62,Assumptions!$A$8:$A$14,0))</f>
@@ -14303,10 +14303,10 @@
         <v>227</v>
       </c>
       <c r="Q62" s="24" t="s">
-        <v>287</v>
+        <v>259</v>
       </c>
       <c r="R62" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14363,13 +14363,13 @@
         <v>0.4167</v>
       </c>
       <c r="P63" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q63" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R63" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14427,7 +14427,7 @@
         <v>0</v>
       </c>
       <c r="P64" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q64" s="24" t="s">
         <v>353</v>
@@ -14490,7 +14490,7 @@
         <v>0.25</v>
       </c>
       <c r="P65" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q65" s="24" t="s">
         <v>355</v>
@@ -14553,7 +14553,7 @@
         <v>0</v>
       </c>
       <c r="P66" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q66" s="24" t="s">
         <v>357</v>
@@ -14620,7 +14620,7 @@
         <v>227</v>
       </c>
       <c r="Q67" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R67" s="2" t="s">
         <v>247</v>
@@ -14810,10 +14810,10 @@
         <v>227</v>
       </c>
       <c r="Q70" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R70" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14876,7 +14876,7 @@
         <v>364</v>
       </c>
       <c r="R71" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14937,7 +14937,7 @@
         <v>227</v>
       </c>
       <c r="Q72" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R72" s="2" t="s">
         <v>229</v>
@@ -15067,7 +15067,7 @@
         <v>369</v>
       </c>
       <c r="R74" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15130,7 +15130,7 @@
         <v>372</v>
       </c>
       <c r="R75" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15193,7 +15193,7 @@
         <v>374</v>
       </c>
       <c r="R76" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15256,7 +15256,7 @@
         <v>377</v>
       </c>
       <c r="R77" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15317,7 +15317,7 @@
         <v>227</v>
       </c>
       <c r="Q78" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R78" s="2" t="s">
         <v>235</v>
@@ -15507,7 +15507,7 @@
         <v>227</v>
       </c>
       <c r="Q81" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R81" s="2" t="s">
         <v>293</v>
@@ -15882,7 +15882,7 @@
         <v>0</v>
       </c>
       <c r="P87" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q87" s="24" t="s">
         <v>395</v>
@@ -15943,7 +15943,7 @@
         <v>0</v>
       </c>
       <c r="P88" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q88" s="24" t="s">
         <v>397</v>
@@ -16004,7 +16004,7 @@
         <v>0</v>
       </c>
       <c r="P89" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q89" s="24" t="s">
         <v>399</v>
@@ -16069,7 +16069,7 @@
         <v>227</v>
       </c>
       <c r="Q90" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R90" s="2" t="s">
         <v>229</v>
@@ -16199,7 +16199,7 @@
         <v>404</v>
       </c>
       <c r="R92" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16262,7 +16262,7 @@
         <v>406</v>
       </c>
       <c r="R93" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16325,7 +16325,7 @@
         <v>408</v>
       </c>
       <c r="R94" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16388,7 +16388,7 @@
         <v>410</v>
       </c>
       <c r="R95" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16449,7 +16449,7 @@
         <v>227</v>
       </c>
       <c r="Q96" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R96" s="2" t="s">
         <v>247</v>
@@ -16639,10 +16639,10 @@
         <v>227</v>
       </c>
       <c r="Q99" s="24" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="R99" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16705,7 +16705,7 @@
         <v>418</v>
       </c>
       <c r="R100" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16766,7 +16766,7 @@
         <v>227</v>
       </c>
       <c r="Q101" s="24" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R101" s="2" t="s">
         <v>235</v>
@@ -16853,22 +16853,22 @@
       </c>
       <c r="F103" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B103,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="G103" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H103" s="21" t="n">
         <f aca="false">F103+G103</f>
-        <v>0.75</v>
+        <v>2</v>
       </c>
       <c r="I103" s="2" t="n">
         <f aca="false">ROUND(H103*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J103" s="2" t="n">
         <f aca="false">ROUND(F103*60,0)</f>
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="K103" s="2" t="n">
         <f aca="false">ROUND(G103*60,0)</f>
@@ -16879,11 +16879,11 @@
       </c>
       <c r="M103" s="22" t="n">
         <f aca="false">F103*IF(L103="CFO",Assumptions!$B$5,Assumptions!$B$4)+G103*Assumptions!$B$5</f>
-        <v>71.25</v>
+        <v>190</v>
       </c>
       <c r="N103" s="16" t="n">
         <f aca="false">F103*INDEX(Assumptions!$B$8:$B$14,MATCH(E103,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="O103" s="16" t="n">
         <f aca="false">G103*INDEX(Assumptions!$B$8:$B$14,MATCH(E103,Assumptions!$A$8:$A$14,0))</f>
@@ -17043,22 +17043,22 @@
       </c>
       <c r="F106" s="16" t="n">
         <f aca="false">IFERROR(INDEX('1099 Oct 30'!$H$5:$H$45,MATCH(B106,'1099 Oct 30'!$A$5:$A$45,0)),0)</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="G106" s="15" t="n">
         <v>0</v>
       </c>
       <c r="H106" s="21" t="n">
         <f aca="false">F106+G106</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="I106" s="2" t="n">
         <f aca="false">ROUND(H106*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="J106" s="2" t="n">
         <f aca="false">ROUND(F106*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="K106" s="2" t="n">
         <f aca="false">ROUND(G106*60,0)</f>
@@ -17069,11 +17069,11 @@
       </c>
       <c r="M106" s="22" t="n">
         <f aca="false">F106*IF(L106="CFO",Assumptions!$B$5,Assumptions!$B$4)+G106*Assumptions!$B$5</f>
-        <v>71.25</v>
+        <v>35.625</v>
       </c>
       <c r="N106" s="16" t="n">
         <f aca="false">F106*INDEX(Assumptions!$B$8:$B$14,MATCH(E106,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="O106" s="16" t="n">
         <f aca="false">G106*INDEX(Assumptions!$B$8:$B$14,MATCH(E106,Assumptions!$A$8:$A$14,0))</f>
@@ -17210,7 +17210,7 @@
         <v>227</v>
       </c>
       <c r="Q108" s="24" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R108" s="2" t="s">
         <v>229</v>
@@ -17270,10 +17270,10 @@
         <v>0.25</v>
       </c>
       <c r="P109" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q109" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R109" s="2" t="s">
         <v>229</v>
@@ -17337,7 +17337,7 @@
         <v>227</v>
       </c>
       <c r="Q110" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R110" s="2" t="s">
         <v>229</v>
@@ -17716,7 +17716,7 @@
         <v>227</v>
       </c>
       <c r="Q116" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R116" s="2" t="s">
         <v>229</v>
@@ -17776,10 +17776,10 @@
         <v>0.5</v>
       </c>
       <c r="P117" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q117" s="24" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R117" s="2" t="s">
         <v>229</v>
@@ -17840,7 +17840,7 @@
         <v>0</v>
       </c>
       <c r="P118" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q118" s="24" t="s">
         <v>448</v>
@@ -17903,7 +17903,7 @@
         <v>0.541666666666667</v>
       </c>
       <c r="P119" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q119" s="24" t="s">
         <v>450</v>
@@ -17966,7 +17966,7 @@
         <v>2.8333</v>
       </c>
       <c r="P120" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q120" s="24" t="s">
         <v>452</v>
@@ -18029,7 +18029,7 @@
         <v>0</v>
       </c>
       <c r="P121" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q121" s="24" t="s">
         <v>454</v>
@@ -18092,7 +18092,7 @@
         <v>1.08333333333333</v>
       </c>
       <c r="P122" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q122" s="24" t="s">
         <v>456</v>
@@ -18155,7 +18155,7 @@
         <v>0</v>
       </c>
       <c r="P123" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q123" s="24" t="s">
         <v>458</v>
@@ -18222,7 +18222,7 @@
         <v>227</v>
       </c>
       <c r="Q124" s="24" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="R124" s="2" t="s">
         <v>235</v>
@@ -19111,7 +19111,7 @@
         <v>Includes Month-end 1.3.</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19141,22 +19141,22 @@
       </c>
       <c r="I15" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P15,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="J15" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="21" t="n">
         <f aca="false">I15+J15</f>
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="L15" s="2" t="n">
         <f aca="false">ROUND(K15*60,0)</f>
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="M15" s="22" t="n">
         <f aca="false">I15*Assumptions!$B$4</f>
-        <v>237.5</v>
+        <v>142.5</v>
       </c>
       <c r="N15" s="23" t="s">
         <v>227</v>
@@ -19222,7 +19222,7 @@
         <v>Josephine's Apr–May 2026 closes + allowance for a new person (Valentina's hours not used).</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19333,7 +19333,7 @@
         <v>Josephine's Apr–May 2026 closes + allowance for a new person (Valentina's hours not used). Will become an Airbnb – provisional. Revisit once it converts.</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19588,22 +19588,22 @@
       </c>
       <c r="I23" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P23,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="J23" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K23" s="21" t="n">
         <f aca="false">I23+J23</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="L23" s="2" t="n">
         <f aca="false">ROUND(K23*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="M23" s="22" t="n">
         <f aca="false">I23*Assumptions!$B$4</f>
-        <v>190</v>
+        <v>71.25</v>
       </c>
       <c r="N23" s="23" t="s">
         <v>227</v>
@@ -19726,7 +19726,7 @@
         <v>Includes Month-end 0.7, Payroll 0.4.</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19783,7 +19783,7 @@
         <v>Includes Month-end 0.7, Payroll 0.4.</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19894,7 +19894,7 @@
         <v>Includes Month-end 2.6, Bookkeeping 0.9.</v>
       </c>
       <c r="P28" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19951,7 +19951,7 @@
         <v>Year-end/tax hours Oct 2025–Sep 2026 (0.5h).</v>
       </c>
       <c r="P29" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20746,22 +20746,22 @@
       </c>
       <c r="I44" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P44,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K44" s="21" t="n">
         <f aca="false">I44+J44</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="L44" s="2" t="n">
         <f aca="false">ROUND(K44*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="M44" s="22" t="n">
         <f aca="false">I44*Assumptions!$B$4</f>
-        <v>142.5</v>
+        <v>380</v>
       </c>
       <c r="N44" s="23" t="s">
         <v>227</v>
@@ -20908,22 +20908,22 @@
       </c>
       <c r="I47" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P47,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="J47" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K47" s="21" t="n">
         <f aca="false">I47+J47</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="L47" s="2" t="n">
         <f aca="false">ROUND(K47*60,0)</f>
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="M47" s="22" t="n">
         <f aca="false">I47*Assumptions!$B$4</f>
-        <v>190</v>
+        <v>71.25</v>
       </c>
       <c r="N47" s="23" t="s">
         <v>227</v>
@@ -21939,22 +21939,22 @@
       </c>
       <c r="I66" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P66,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="J66" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K66" s="21" t="n">
         <f aca="false">I66+J66</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="L66" s="2" t="n">
         <f aca="false">ROUND(K66*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="M66" s="22" t="n">
         <f aca="false">I66*Assumptions!$B$4</f>
-        <v>142.5</v>
+        <v>380</v>
       </c>
       <c r="N66" s="23" t="s">
         <v>227</v>
@@ -22883,22 +22883,22 @@
       </c>
       <c r="I88" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P88,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="J88" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K88" s="21" t="n">
         <f aca="false">I88+J88</f>
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="L88" s="2" t="n">
         <f aca="false">ROUND(K88*60,0)</f>
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="M88" s="22" t="n">
         <f aca="false">I88*Assumptions!$B$4</f>
-        <v>71.25</v>
+        <v>35.625</v>
       </c>
       <c r="N88" s="23" t="s">
         <v>227</v>
@@ -26693,22 +26693,22 @@
       </c>
       <c r="I157" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P157,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="J157" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K157" s="21" t="n">
         <f aca="false">I157+J157</f>
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="L157" s="2" t="n">
         <f aca="false">ROUND(K157*60,0)</f>
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="M157" s="22" t="n">
         <f aca="false">I157*Assumptions!$B$4</f>
-        <v>142.5</v>
+        <v>380</v>
       </c>
       <c r="N157" s="23" t="s">
         <v>227</v>
@@ -26861,22 +26861,22 @@
       </c>
       <c r="I160" s="16" t="n">
         <f aca="false">INDEX('1099 Oct 30'!$F$5:$F$45,MATCH(P160,'1099 Oct 30'!$A$5:$A$45,0))</f>
-        <v>1.125</v>
+        <v>0.5625</v>
       </c>
       <c r="J160" s="15" t="n">
         <v>0</v>
       </c>
       <c r="K160" s="21" t="n">
         <f aca="false">I160+J160</f>
-        <v>1.125</v>
+        <v>0.5625</v>
       </c>
       <c r="L160" s="2" t="n">
         <f aca="false">ROUND(K160*60,0)</f>
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="M160" s="22" t="n">
         <f aca="false">I160*Assumptions!$B$4</f>
-        <v>106.875</v>
+        <v>53.4375</v>
       </c>
       <c r="N160" s="23" t="s">
         <v>227</v>
@@ -28254,7 +28254,7 @@
       <c r="H186" s="2"/>
       <c r="I186" s="4" t="n">
         <f aca="false">SUM(I2:I184)</f>
-        <v>537.8333</v>
+        <v>540.8958</v>
       </c>
       <c r="J186" s="4" t="n">
         <f aca="false">SUM(J2:J184)</f>
@@ -28262,15 +28262,15 @@
       </c>
       <c r="K186" s="4" t="n">
         <f aca="false">SUM(K2:K184)</f>
-        <v>593.8333</v>
+        <v>596.8958</v>
       </c>
       <c r="L186" s="4" t="n">
         <f aca="false">SUM(L2:L184)</f>
-        <v>35634</v>
+        <v>35818</v>
       </c>
       <c r="M186" s="32" t="n">
         <f aca="false">SUM(M2:M184)</f>
-        <v>72314.606</v>
+        <v>72605.5435</v>
       </c>
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>
@@ -28452,7 +28452,7 @@
       </c>
       <c r="B9" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A9)</f>
-        <v>1.66666666666667</v>
+        <v>1.5</v>
       </c>
       <c r="C9" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A9)</f>
@@ -28460,7 +28460,7 @@
       </c>
       <c r="D9" s="35" t="n">
         <f aca="false">B9+C9</f>
-        <v>2.24996666666667</v>
+        <v>2.0833</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>232</v>
@@ -28484,7 +28484,7 @@
         <v>1.125</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F10" s="2"/>
     </row>
@@ -28505,7 +28505,7 @@
         <v>1.7083</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>549</v>
@@ -28517,7 +28517,7 @@
       </c>
       <c r="B12" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A12)</f>
-        <v>25.9164916666667</v>
+        <v>25.499825</v>
       </c>
       <c r="C12" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A12)</f>
@@ -28525,7 +28525,7 @@
       </c>
       <c r="D12" s="35" t="n">
         <f aca="false">B12+C12</f>
-        <v>26.2497916666667</v>
+        <v>25.833125</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>232</v>
@@ -28643,7 +28643,7 @@
       </c>
       <c r="B18" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A18)</f>
-        <v>2.6667</v>
+        <v>3.08336666666667</v>
       </c>
       <c r="C18" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A18)</f>
@@ -28651,7 +28651,7 @@
       </c>
       <c r="D18" s="35" t="n">
         <f aca="false">B18+C18</f>
-        <v>3.5</v>
+        <v>3.91666666666667</v>
       </c>
       <c r="E18" s="25" t="s">
         <v>232</v>
@@ -28664,7 +28664,7 @@
       </c>
       <c r="B19" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A19)</f>
-        <v>7.74996666666667</v>
+        <v>7.3333</v>
       </c>
       <c r="C19" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A19)</f>
@@ -28672,7 +28672,7 @@
       </c>
       <c r="D19" s="35" t="n">
         <f aca="false">B19+C19</f>
-        <v>9.49996666666667</v>
+        <v>9.0833</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>232</v>
@@ -28719,7 +28719,7 @@
         <v>1.2083</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F21" s="2"/>
     </row>
@@ -28784,7 +28784,7 @@
         <v>7.5</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>551</v>
@@ -28819,7 +28819,7 @@
       </c>
       <c r="B26" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A26)</f>
-        <v>0.25</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="C26" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A26)</f>
@@ -28827,7 +28827,7 @@
       </c>
       <c r="D26" s="35" t="n">
         <f aca="false">B26+C26</f>
-        <v>0.25</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="E26" s="23" t="s">
         <v>227</v>
@@ -28884,7 +28884,7 @@
       </c>
       <c r="B29" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A29)</f>
-        <v>0.75</v>
+        <v>0.625</v>
       </c>
       <c r="C29" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A29)</f>
@@ -28892,10 +28892,10 @@
       </c>
       <c r="D29" s="35" t="n">
         <f aca="false">B29+C29</f>
-        <v>1.1667</v>
+        <v>1.0417</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F29" s="2"/>
     </row>
@@ -28916,7 +28916,7 @@
         <v>3.125</v>
       </c>
       <c r="E30" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>553</v>
@@ -29088,7 +29088,7 @@
         <v>8.311775</v>
       </c>
       <c r="E38" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F38" s="2"/>
     </row>
@@ -29205,7 +29205,7 @@
       </c>
       <c r="B44" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A44)</f>
-        <v>2.125</v>
+        <v>2.54166666666667</v>
       </c>
       <c r="C44" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A44)</f>
@@ -29213,7 +29213,7 @@
       </c>
       <c r="D44" s="35" t="n">
         <f aca="false">B44+C44</f>
-        <v>2.125</v>
+        <v>2.54166666666667</v>
       </c>
       <c r="E44" s="28" t="s">
         <v>376</v>
@@ -29228,7 +29228,7 @@
       </c>
       <c r="B45" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A45)</f>
-        <v>1.5833</v>
+        <v>1.4583</v>
       </c>
       <c r="C45" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A45)</f>
@@ -29236,7 +29236,7 @@
       </c>
       <c r="D45" s="35" t="n">
         <f aca="false">B45+C45</f>
-        <v>2.3333</v>
+        <v>2.2083</v>
       </c>
       <c r="E45" s="28" t="s">
         <v>312</v>
@@ -29262,7 +29262,7 @@
         <v>1.125</v>
       </c>
       <c r="E46" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F46" s="2"/>
     </row>
@@ -29304,7 +29304,7 @@
         <v>1.25</v>
       </c>
       <c r="E48" s="26" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F48" s="2"/>
     </row>
@@ -29325,7 +29325,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>557</v>
@@ -29798,7 +29798,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>5.5</v>
@@ -30592,7 +30592,7 @@
         <v>0.75</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30951,7 +30951,7 @@
         <v>4.75</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31052,7 +31052,7 @@
         <v>2.5</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31575,7 +31575,7 @@
         <v>12.2</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31803,7 +31803,7 @@
         <v>17.6</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31920,7 +31920,7 @@
         <v>1</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32144,7 +32144,7 @@
         <v>7.25</v>
       </c>
       <c r="O64" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32776,7 +32776,7 @@
         <v>1</v>
       </c>
       <c r="O82" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32869,7 +32869,7 @@
       <c r="M85" s="36"/>
       <c r="N85" s="36"/>
       <c r="O85" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33269,7 +33269,7 @@
       </c>
       <c r="N97" s="36"/>
       <c r="O97" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33497,7 +33497,7 @@
         <v>50.85</v>
       </c>
       <c r="O103" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34052,7 +34052,7 @@
         <v>3.3</v>
       </c>
       <c r="O118" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34280,7 +34280,7 @@
         <v>7</v>
       </c>
       <c r="O124" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Review: use logged time per close, no 0.7 floor; 0.5h placeholder where none logged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRgGtk6aohavQBQTYDwapz
</commit_message>
<xml_diff>
--- a/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
+++ b/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
@@ -749,7 +749,7 @@
     <t xml:space="preserve">Accounting</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 0.5. Review = 1.25h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 0.5. Review = 1.25h as logged (only 2 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">15650 Northsight LLC|Sales tax|Quarterly Sales Tax Filing - Onyx Prepares the Returns for Client|Quarterly</t>
@@ -893,7 +893,7 @@
     <t xml:space="preserve">Barrett Living Trust|Accounting|Month End Close|Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 2.6, Bookkeeping 0.9. Review = 1.10h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 2.6, Bookkeeping 0.9. Review = 1.10h as logged (only 2 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">BeckShar Development LLC|1099|1099 Quarterly Review|1099</t>
@@ -923,7 +923,7 @@
     <t xml:space="preserve">BeckShar LLC|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h as logged (only 2 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">Building and Development Professionals LLC|1099|1099 Quarterly Review|1099</t>
@@ -932,7 +932,7 @@
     <t xml:space="preserve">Building and Development Professionals LLC|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 0.5, CFO advisory 1.9. Review = 0.7h standard (no close reviews found in Harvest).</t>
+    <t xml:space="preserve">Includes Month-end 0.5, CFO advisory 1.9. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</t>
   </si>
   <si>
     <t xml:space="preserve">Capital Financial LLC|1099|1099 Quarterly Review|1099</t>
@@ -1049,7 +1049,7 @@
     <t xml:space="preserve">GAV Enterprises Inc|Accounting|Quarter End Close|Quarterly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">International Alliance Group LLC|1099|1099 Quarterly Review|1099</t>
@@ -1172,7 +1172,7 @@
     <t xml:space="preserve">Low</t>
   </si>
   <si>
-    <t xml:space="preserve">SUGGESTED – no recurring month-end item in the Oct list (only the July clean-up). Payroll takeover in progress (Paychex/401k/PFML); tax audit budgeted separately. Confirm payroll is ongoing. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">SUGGESTED – no recurring month-end item in the Oct list (only the July clean-up). Payroll takeover in progress (Paychex/401k/PFML); tax audit budgeted separately. Confirm payroll is ongoing. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">Newport Classic Cars LLC|1099|1099 Quarterly Review|1099</t>
@@ -1220,7 +1220,7 @@
     <t xml:space="preserve">Paradise Village LLC|Accounting|Quarter End Close|Quarterly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 1.0. Review = 1.00h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 1.0. Review = 1.00h as logged (only 2 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">Phil Tavasci Companies|Bookkeeping|Daily Chase Fraud Review|Daily</t>
@@ -1265,7 +1265,7 @@
     <t xml:space="preserve">Prestige Arms Worldwide|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</t>
+    <t xml:space="preserve">Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</t>
   </si>
   <si>
     <t xml:space="preserve">Prestige Arms Worldwide|Sales tax|Sales Tax Filing - Onyx Prepares the Returns for Client|Monthly</t>
@@ -1322,7 +1322,7 @@
     <t xml:space="preserve">Southwest Rents Inc|Monthly Financials|Month End Close|Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.7h standard (no close reviews found in Harvest).</t>
+    <t xml:space="preserve">Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.5h placeholder (no close reviews found in Harvest) – check.</t>
   </si>
   <si>
     <t xml:space="preserve">T5 Family Holdings LLC|1099|1099 Quarterly Review|1099</t>
@@ -1427,7 +1427,7 @@
     <t xml:space="preserve">Young Wealth Management PLLC|Accounting|Quarter End Close|Quarterly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 6.5, Payroll 1.2. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</t>
+    <t xml:space="preserve">Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</t>
   </si>
   <si>
     <t xml:space="preserve">Work Title</t>
@@ -3771,19 +3771,19 @@
       </c>
       <c r="D37" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F33*60,0)/1440</f>
-        <v>0.107638888888889</v>
+        <v>0.114583333333333</v>
       </c>
       <c r="E37" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F33*IF(H37="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>646</v>
+        <v>688</v>
       </c>
       <c r="F37" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G33*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="G37" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G33*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="H37" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L33</f>
@@ -4329,19 +4329,19 @@
       </c>
       <c r="D55" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F52*60,0)/1440</f>
-        <v>0.756944444444444</v>
+        <v>0.774305555555556</v>
       </c>
       <c r="E55" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F52*IF(H55="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>1726</v>
+        <v>1765</v>
       </c>
       <c r="F55" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G52*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0104166666666667</v>
       </c>
       <c r="G55" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G52*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="H55" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L52</f>
@@ -4825,19 +4825,19 @@
       </c>
       <c r="D71" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F77*60,0)/1440</f>
-        <v>0.177083333333333</v>
+        <v>0.194444444444444</v>
       </c>
       <c r="E71" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F77*IF(H71="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>404</v>
+        <v>443</v>
       </c>
       <c r="F71" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G77*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0104166666666667</v>
       </c>
       <c r="G71" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G77*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="H71" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L77</f>
@@ -5360,11 +5360,11 @@
       </c>
       <c r="F88" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G94*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="G88" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G94*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="H88" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L94</f>
@@ -5662,19 +5662,19 @@
       </c>
       <c r="D98" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F105*60,0)/1440</f>
-        <v>0.0347222222222222</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="E98" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F105*IF(H98="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="F98" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G105*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="G98" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G105*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="H98" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L105</f>
@@ -6282,19 +6282,19 @@
       </c>
       <c r="D118" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F125*60,0)/1440</f>
-        <v>0.302083333333333</v>
+        <v>0.315972222222222</v>
       </c>
       <c r="E118" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!F125*IF(H118="CFO",Assumptions!$B$5,Assumptions!$B$4),0)</f>
-        <v>689</v>
+        <v>720</v>
       </c>
       <c r="F118" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G125*60,0)/1440</f>
-        <v>0.0291666666666667</v>
+        <v>0.0145833333333333</v>
       </c>
       <c r="G118" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G125*Assumptions!$B$5,0)</f>
-        <v>175</v>
+        <v>88</v>
       </c>
       <c r="H118" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L125</f>
@@ -12636,41 +12636,41 @@
         <v>15</v>
       </c>
       <c r="F33" s="15" t="n">
-        <v>2.5833</v>
+        <v>2.75</v>
       </c>
       <c r="G33" s="15" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="H33" s="21" t="n">
         <f aca="false">F33+G33</f>
-        <v>3.2833</v>
+        <v>3.25</v>
       </c>
       <c r="I33" s="2" t="n">
         <f aca="false">ROUND(H33*60,0)</f>
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J33" s="2" t="n">
         <f aca="false">ROUND(F33*60,0)</f>
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="K33" s="2" t="n">
         <f aca="false">ROUND(G33*60,0)</f>
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L33" s="9" t="s">
         <v>185</v>
       </c>
       <c r="M33" s="22" t="n">
         <f aca="false">F33*IF(L33="CFO",Assumptions!$B$5,Assumptions!$B$4)+G33*Assumptions!$B$5</f>
-        <v>820.825</v>
+        <v>812.5</v>
       </c>
       <c r="N33" s="16" t="n">
         <f aca="false">F33*INDEX(Assumptions!$B$8:$B$14,MATCH(E33,Assumptions!$A$8:$A$14,0))</f>
-        <v>2.5833</v>
+        <v>2.75</v>
       </c>
       <c r="O33" s="16" t="n">
         <f aca="false">G33*INDEX(Assumptions!$B$8:$B$14,MATCH(E33,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="P33" s="25" t="s">
         <v>232</v>
@@ -13811,41 +13811,41 @@
         <v>13</v>
       </c>
       <c r="F52" s="15" t="n">
-        <v>18.1667</v>
+        <v>18.5833</v>
       </c>
       <c r="G52" s="15" t="n">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="H52" s="21" t="n">
         <f aca="false">F52+G52</f>
-        <v>18.8667</v>
+        <v>18.8333</v>
       </c>
       <c r="I52" s="2" t="n">
         <f aca="false">ROUND(H52*60,0)</f>
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="J52" s="2" t="n">
         <f aca="false">ROUND(F52*60,0)</f>
-        <v>1090</v>
+        <v>1115</v>
       </c>
       <c r="K52" s="2" t="n">
         <f aca="false">ROUND(G52*60,0)</f>
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="L52" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M52" s="22" t="n">
         <f aca="false">F52*IF(L52="CFO",Assumptions!$B$5,Assumptions!$B$4)+G52*Assumptions!$B$5</f>
-        <v>1900.8365</v>
+        <v>1827.9135</v>
       </c>
       <c r="N52" s="16" t="n">
         <f aca="false">F52*INDEX(Assumptions!$B$8:$B$14,MATCH(E52,Assumptions!$A$8:$A$14,0))</f>
-        <v>6.05556666666667</v>
+        <v>6.19443333333333</v>
       </c>
       <c r="O52" s="16" t="n">
         <f aca="false">G52*INDEX(Assumptions!$B$8:$B$14,MATCH(E52,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.233333333333333</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="P52" s="25" t="s">
         <v>232</v>
@@ -15131,41 +15131,41 @@
         <v>15</v>
       </c>
       <c r="F77" s="15" t="n">
-        <v>4.25</v>
+        <v>4.6667</v>
       </c>
       <c r="G77" s="15" t="n">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="H77" s="21" t="n">
         <f aca="false">F77+G77</f>
-        <v>4.95</v>
+        <v>4.9167</v>
       </c>
       <c r="I77" s="2" t="n">
         <f aca="false">ROUND(H77*60,0)</f>
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J77" s="2" t="n">
         <f aca="false">ROUND(F77*60,0)</f>
-        <v>255</v>
+        <v>280</v>
       </c>
       <c r="K77" s="2" t="n">
         <f aca="false">ROUND(G77*60,0)</f>
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="L77" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M77" s="22" t="n">
         <f aca="false">F77*IF(L77="CFO",Assumptions!$B$5,Assumptions!$B$4)+G77*Assumptions!$B$5</f>
-        <v>578.75</v>
+        <v>505.8365</v>
       </c>
       <c r="N77" s="16" t="n">
         <f aca="false">F77*INDEX(Assumptions!$B$8:$B$14,MATCH(E77,Assumptions!$A$8:$A$14,0))</f>
-        <v>4.25</v>
+        <v>4.6667</v>
       </c>
       <c r="O77" s="16" t="n">
         <f aca="false">G77*INDEX(Assumptions!$B$8:$B$14,MATCH(E77,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="P77" s="28" t="s">
         <v>378</v>
@@ -16203,15 +16203,15 @@
         <v>1</v>
       </c>
       <c r="G94" s="15" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="H94" s="21" t="n">
         <f aca="false">F94+G94</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="I94" s="2" t="n">
         <f aca="false">ROUND(H94*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="J94" s="2" t="n">
         <f aca="false">ROUND(F94*60,0)</f>
@@ -16219,14 +16219,14 @@
       </c>
       <c r="K94" s="2" t="n">
         <f aca="false">ROUND(G94*60,0)</f>
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L94" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M94" s="22" t="n">
         <f aca="false">F94*IF(L94="CFO",Assumptions!$B$5,Assumptions!$B$4)+G94*Assumptions!$B$5</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N94" s="16" t="n">
         <f aca="false">F94*INDEX(Assumptions!$B$8:$B$14,MATCH(E94,Assumptions!$A$8:$A$14,0))</f>
@@ -16234,7 +16234,7 @@
       </c>
       <c r="O94" s="16" t="n">
         <f aca="false">G94*INDEX(Assumptions!$B$8:$B$14,MATCH(E94,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="P94" s="23" t="s">
         <v>227</v>
@@ -16897,41 +16897,41 @@
         <v>15</v>
       </c>
       <c r="F105" s="15" t="n">
-        <v>0.8333</v>
+        <v>1</v>
       </c>
       <c r="G105" s="15" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="H105" s="21" t="n">
         <f aca="false">F105+G105</f>
-        <v>1.5333</v>
+        <v>1.5</v>
       </c>
       <c r="I105" s="2" t="n">
         <f aca="false">ROUND(H105*60,0)</f>
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J105" s="2" t="n">
         <f aca="false">ROUND(F105*60,0)</f>
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K105" s="2" t="n">
         <f aca="false">ROUND(G105*60,0)</f>
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L105" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M105" s="22" t="n">
         <f aca="false">F105*IF(L105="CFO",Assumptions!$B$5,Assumptions!$B$4)+G105*Assumptions!$B$5</f>
-        <v>254.1635</v>
+        <v>220</v>
       </c>
       <c r="N105" s="16" t="n">
         <f aca="false">F105*INDEX(Assumptions!$B$8:$B$14,MATCH(E105,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.8333</v>
+        <v>1</v>
       </c>
       <c r="O105" s="16" t="n">
         <f aca="false">G105*INDEX(Assumptions!$B$8:$B$14,MATCH(E105,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="P105" s="28" t="s">
         <v>378</v>
@@ -18163,41 +18163,41 @@
         <v>13</v>
       </c>
       <c r="F125" s="15" t="n">
-        <v>7.25</v>
+        <v>7.5833</v>
       </c>
       <c r="G125" s="15" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="H125" s="21" t="n">
         <f aca="false">F125+G125</f>
-        <v>7.95</v>
+        <v>7.9333</v>
       </c>
       <c r="I125" s="2" t="n">
         <f aca="false">ROUND(H125*60,0)</f>
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="J125" s="2" t="n">
         <f aca="false">ROUND(F125*60,0)</f>
-        <v>435</v>
+        <v>455</v>
       </c>
       <c r="K125" s="2" t="n">
         <f aca="false">ROUND(G125*60,0)</f>
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="L125" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M125" s="22" t="n">
         <f aca="false">F125*IF(L125="CFO",Assumptions!$B$5,Assumptions!$B$4)+G125*Assumptions!$B$5</f>
-        <v>863.75</v>
+        <v>807.9135</v>
       </c>
       <c r="N125" s="16" t="n">
         <f aca="false">F125*INDEX(Assumptions!$B$8:$B$14,MATCH(E125,Assumptions!$A$8:$A$14,0))</f>
-        <v>2.41666666666667</v>
+        <v>2.52776666666667</v>
       </c>
       <c r="O125" s="16" t="n">
         <f aca="false">G125*INDEX(Assumptions!$B$8:$B$14,MATCH(E125,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.233333333333333</v>
+        <v>0.116666666666667</v>
       </c>
       <c r="P125" s="28" t="s">
         <v>314</v>
@@ -18522,7 +18522,7 @@
       </c>
       <c r="O5" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P5,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 0.5. Review = 1.25h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 0.5. Review = 1.25h as logged (only 2 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>236</v>
@@ -19809,7 +19809,7 @@
       </c>
       <c r="O28" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P28,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 2.6, Bookkeeping 0.9. Review = 1.10h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 2.6, Bookkeeping 0.9. Review = 1.10h as logged (only 2 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>285</v>
@@ -20310,7 +20310,7 @@
       </c>
       <c r="O37" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P37,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h as logged (only 2 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P37" s="2" t="s">
         <v>295</v>
@@ -20367,7 +20367,7 @@
       </c>
       <c r="O38" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P38,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 1.2, Bookkeeping 0.5, Payroll 1.3, Sales tax 0.8. Review = 1.25h as logged (only 2 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>295</v>
@@ -20607,23 +20607,23 @@
       </c>
       <c r="I43" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P43,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>2.5833</v>
+        <v>2.75</v>
       </c>
       <c r="J43" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P43,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K43" s="21" t="n">
         <f aca="false">I43+J43</f>
-        <v>3.2833</v>
+        <v>3.25</v>
       </c>
       <c r="L43" s="2" t="n">
         <f aca="false">ROUND(K43*60,0)</f>
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="M43" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P43,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>820.825</v>
+        <v>812.5</v>
       </c>
       <c r="N43" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P43,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -20631,7 +20631,7 @@
       </c>
       <c r="O43" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P43,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 0.5, CFO advisory 1.9. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Includes Month-end 0.5, CFO advisory 1.9. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>298</v>
@@ -21968,23 +21968,23 @@
       </c>
       <c r="I68" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>18.1667</v>
+        <v>18.5833</v>
       </c>
       <c r="J68" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="K68" s="21" t="n">
         <f aca="false">I68+J68</f>
-        <v>18.8667</v>
+        <v>18.8333</v>
       </c>
       <c r="L68" s="2" t="n">
         <f aca="false">ROUND(K68*60,0)</f>
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="M68" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>1900.8365</v>
+        <v>1827.9135</v>
       </c>
       <c r="N68" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -21992,7 +21992,7 @@
       </c>
       <c r="O68" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P68" s="2" t="s">
         <v>337</v>
@@ -24430,7 +24430,7 @@
       </c>
       <c r="O117" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P117,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 1.0. Review = 1.00h (only 2 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 1.0. Review = 1.00h as logged (only 2 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P117" s="2" t="s">
         <v>394</v>
@@ -25079,19 +25079,19 @@
       </c>
       <c r="J129" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P129,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K129" s="21" t="n">
         <f aca="false">I129+J129</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L129" s="2" t="n">
         <f aca="false">ROUND(K129*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M129" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P129,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N129" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P129,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25099,7 +25099,7 @@
       </c>
       <c r="O129" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P129,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P129" s="2" t="s">
         <v>409</v>
@@ -25190,19 +25190,19 @@
       </c>
       <c r="J131" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P131,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K131" s="21" t="n">
         <f aca="false">I131+J131</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L131" s="2" t="n">
         <f aca="false">ROUND(K131*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M131" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P131,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N131" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P131,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25210,7 +25210,7 @@
       </c>
       <c r="O131" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P131,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P131" s="2" t="s">
         <v>409</v>
@@ -25247,19 +25247,19 @@
       </c>
       <c r="J132" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P132,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K132" s="21" t="n">
         <f aca="false">I132+J132</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L132" s="2" t="n">
         <f aca="false">ROUND(K132*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M132" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P132,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N132" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P132,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25267,7 +25267,7 @@
       </c>
       <c r="O132" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P132,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P132" s="2" t="s">
         <v>409</v>
@@ -25304,19 +25304,19 @@
       </c>
       <c r="J133" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P133,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K133" s="21" t="n">
         <f aca="false">I133+J133</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L133" s="2" t="n">
         <f aca="false">ROUND(K133*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M133" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P133,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N133" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P133,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25324,7 +25324,7 @@
       </c>
       <c r="O133" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P133,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P133" s="2" t="s">
         <v>409</v>
@@ -25361,19 +25361,19 @@
       </c>
       <c r="J134" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P134,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K134" s="21" t="n">
         <f aca="false">I134+J134</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L134" s="2" t="n">
         <f aca="false">ROUND(K134*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M134" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P134,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N134" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P134,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25381,7 +25381,7 @@
       </c>
       <c r="O134" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P134,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P134" s="2" t="s">
         <v>409</v>
@@ -25418,19 +25418,19 @@
       </c>
       <c r="J135" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P135,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K135" s="21" t="n">
         <f aca="false">I135+J135</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L135" s="2" t="n">
         <f aca="false">ROUND(K135*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M135" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P135,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N135" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P135,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25438,7 +25438,7 @@
       </c>
       <c r="O135" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P135,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P135" s="2" t="s">
         <v>409</v>
@@ -25475,19 +25475,19 @@
       </c>
       <c r="J136" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P136,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K136" s="21" t="n">
         <f aca="false">I136+J136</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L136" s="2" t="n">
         <f aca="false">ROUND(K136*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M136" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P136,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N136" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P136,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25495,7 +25495,7 @@
       </c>
       <c r="O136" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P136,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P136" s="2" t="s">
         <v>409</v>
@@ -25532,19 +25532,19 @@
       </c>
       <c r="J137" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P137,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K137" s="21" t="n">
         <f aca="false">I137+J137</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L137" s="2" t="n">
         <f aca="false">ROUND(K137*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M137" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P137,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N137" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P137,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25552,7 +25552,7 @@
       </c>
       <c r="O137" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P137,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P137" s="2" t="s">
         <v>409</v>
@@ -25589,19 +25589,19 @@
       </c>
       <c r="J138" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P138,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K138" s="21" t="n">
         <f aca="false">I138+J138</f>
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L138" s="2" t="n">
         <f aca="false">ROUND(K138*60,0)</f>
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M138" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P138,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="N138" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P138,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -25609,7 +25609,7 @@
       </c>
       <c r="O138" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P138,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Little recent history (backlog not yet worked). Close set at 1.0h from 2025 pattern, adjusted for contractor under-recording. Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P138" s="2" t="s">
         <v>409</v>
@@ -26350,23 +26350,23 @@
       </c>
       <c r="I152" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P152,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.8333</v>
+        <v>1</v>
       </c>
       <c r="J152" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P152,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K152" s="21" t="n">
         <f aca="false">I152+J152</f>
-        <v>1.5333</v>
+        <v>1.5</v>
       </c>
       <c r="L152" s="2" t="n">
         <f aca="false">ROUND(K152*60,0)</f>
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="M152" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P152,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>254.1635</v>
+        <v>220</v>
       </c>
       <c r="N152" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P152,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -26374,7 +26374,7 @@
       </c>
       <c r="O152" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P152,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P152" s="2" t="s">
         <v>428</v>
@@ -26560,23 +26560,23 @@
       </c>
       <c r="I156" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P156,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.8333</v>
+        <v>1</v>
       </c>
       <c r="J156" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P156,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="K156" s="21" t="n">
         <f aca="false">I156+J156</f>
-        <v>1.5333</v>
+        <v>1.5</v>
       </c>
       <c r="L156" s="2" t="n">
         <f aca="false">ROUND(K156*60,0)</f>
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="M156" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P156,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>254.1635</v>
+        <v>220</v>
       </c>
       <c r="N156" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P156,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -26584,7 +26584,7 @@
       </c>
       <c r="O156" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P156,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.7h standard (no close reviews found in Harvest).</v>
+        <v>Includes Month-end 0.2, Bookkeeping 0.5, Sales tax 0.2, CFO advisory 0.6. Catch-up still underway; steady level uncertain. Backlog closes carry the remaining catch-up (~15–20h). Review = 0.5h placeholder (no close reviews found in Harvest) – check.</v>
       </c>
       <c r="P156" s="2" t="s">
         <v>428</v>
@@ -28006,23 +28006,23 @@
       </c>
       <c r="I182" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>7.25</v>
+        <v>7.5833</v>
       </c>
       <c r="J182" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="K182" s="21" t="n">
         <f aca="false">I182+J182</f>
-        <v>7.95</v>
+        <v>7.9333</v>
       </c>
       <c r="L182" s="2" t="n">
         <f aca="false">ROUND(K182*60,0)</f>
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="M182" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>863.75</v>
+        <v>807.9135</v>
       </c>
       <c r="N182" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -28030,7 +28030,7 @@
       </c>
       <c r="O182" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P182" s="2" t="s">
         <v>463</v>
@@ -28063,23 +28063,23 @@
       </c>
       <c r="I183" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$F$2:$F$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>7.25</v>
+        <v>7.5833</v>
       </c>
       <c r="J183" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="K183" s="21" t="n">
         <f aca="false">I183+J183</f>
-        <v>7.95</v>
+        <v>7.9333</v>
       </c>
       <c r="L183" s="2" t="n">
         <f aca="false">ROUND(K183*60,0)</f>
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="M183" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>863.75</v>
+        <v>807.9135</v>
       </c>
       <c r="N183" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -28087,7 +28087,7 @@
       </c>
       <c r="O183" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.70h (only 1 reviewed close(s) in Harvest; 0.7h standard applied as minimum).</v>
+        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</v>
       </c>
       <c r="P183" s="2" t="s">
         <v>463</v>
@@ -28178,23 +28178,23 @@
       <c r="H186" s="2"/>
       <c r="I186" s="4" t="n">
         <f aca="false">SUM(I2:I184)</f>
-        <v>549.146</v>
+        <v>550.7293</v>
       </c>
       <c r="J186" s="4" t="n">
         <f aca="false">SUM(J2:J184)</f>
-        <v>55.3831</v>
+        <v>51.8331</v>
       </c>
       <c r="K186" s="4" t="n">
         <f aca="false">SUM(K2:K184)</f>
-        <v>604.5291</v>
+        <v>602.5624</v>
       </c>
       <c r="L186" s="4" t="n">
         <f aca="false">SUM(L2:L184)</f>
-        <v>36276</v>
+        <v>36158</v>
       </c>
       <c r="M186" s="32" t="n">
         <f aca="false">SUM(M2:M184)</f>
-        <v>73092.9835</v>
+        <v>72381.7355</v>
       </c>
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>
@@ -28567,15 +28567,15 @@
       </c>
       <c r="B18" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A18)</f>
-        <v>3.24996666666667</v>
+        <v>3.41666666666667</v>
       </c>
       <c r="C18" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A18)</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D18" s="35" t="n">
         <f aca="false">B18+C18</f>
-        <v>3.94996666666667</v>
+        <v>3.91666666666667</v>
       </c>
       <c r="E18" s="25" t="s">
         <v>232</v>
@@ -28764,15 +28764,15 @@
       </c>
       <c r="B27" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A27)</f>
-        <v>6.36111666666667</v>
+        <v>6.49998333333333</v>
       </c>
       <c r="C27" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A27)</f>
-        <v>0.233333333333333</v>
+        <v>0.0833333333333333</v>
       </c>
       <c r="D27" s="35" t="n">
         <f aca="false">B27+C27</f>
-        <v>6.59445</v>
+        <v>6.58331666666667</v>
       </c>
       <c r="E27" s="25" t="s">
         <v>232</v>
@@ -28915,15 +28915,15 @@
       </c>
       <c r="B34" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A34)</f>
-        <v>7.625</v>
+        <v>8.0417</v>
       </c>
       <c r="C34" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A34)</f>
-        <v>1.60285</v>
+        <v>1.15285</v>
       </c>
       <c r="D34" s="35" t="n">
         <f aca="false">B34+C34</f>
-        <v>9.22785</v>
+        <v>9.19455</v>
       </c>
       <c r="E34" s="28" t="s">
         <v>378</v>
@@ -29047,11 +29047,11 @@
       </c>
       <c r="C40" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A40)</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D40" s="35" t="n">
         <f aca="false">B40+C40</f>
-        <v>2.102775</v>
+        <v>1.902775</v>
       </c>
       <c r="E40" s="25" t="s">
         <v>232</v>
@@ -29129,15 +29129,15 @@
       </c>
       <c r="B44" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A44)</f>
-        <v>1.87496666666667</v>
+        <v>2.04166666666667</v>
       </c>
       <c r="C44" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A44)</f>
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D44" s="35" t="n">
         <f aca="false">B44+C44</f>
-        <v>2.57496666666667</v>
+        <v>2.54166666666667</v>
       </c>
       <c r="E44" s="28" t="s">
         <v>378</v>
@@ -29261,15 +29261,15 @@
       </c>
       <c r="B50" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$N$2:$N$125,'Recurring Budgets'!$B$2:$B$125,A50)</f>
-        <v>2.66666666666667</v>
+        <v>2.77776666666667</v>
       </c>
       <c r="C50" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A50)</f>
-        <v>0.233333333333333</v>
+        <v>0.116666666666667</v>
       </c>
       <c r="D50" s="35" t="n">
         <f aca="false">B50+C50</f>
-        <v>2.9</v>
+        <v>2.89443333333333</v>
       </c>
       <c r="E50" s="28" t="s">
         <v>314</v>
@@ -29282,15 +29282,15 @@
       </c>
       <c r="B51" s="19" t="n">
         <f aca="false">SUM(B4:B50)</f>
-        <v>274.200525</v>
+        <v>275.200591666667</v>
       </c>
       <c r="C51" s="19" t="n">
         <f aca="false">SUM(C4:C50)</f>
-        <v>33.78595</v>
+        <v>32.4692833333333</v>
       </c>
       <c r="D51" s="19" t="n">
         <f aca="false">SUM(D4:D50)</f>
-        <v>307.986475</v>
+        <v>307.669875</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -29335,15 +29335,15 @@
       </c>
       <c r="B55" s="4" t="n">
         <f aca="false">B51+B54</f>
-        <v>284.200525</v>
+        <v>285.200591666667</v>
       </c>
       <c r="C55" s="4" t="n">
         <f aca="false">C51+C53</f>
-        <v>58.78595</v>
+        <v>57.4692833333333</v>
       </c>
       <c r="D55" s="4" t="n">
         <f aca="false">B55+C55</f>
-        <v>342.986475</v>
+        <v>342.669875</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>

</xml_diff>

<commit_message>
Mountain Trade month-end review set to 0:50 (CYMA system)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRgGtk6aohavQBQTYDwapz
</commit_message>
<xml_diff>
--- a/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
+++ b/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
@@ -1172,7 +1172,7 @@
     <t xml:space="preserve">Low</t>
   </si>
   <si>
-    <t xml:space="preserve">SUGGESTED – no recurring month-end item in the Oct list (only the July clean-up). Payroll takeover in progress (Paychex/401k/PFML); tax audit budgeted separately. Confirm payroll is ongoing. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</t>
+    <t xml:space="preserve">SUGGESTED – no recurring month-end item in the Oct list (only the July clean-up). Payroll takeover in progress (Paychex/401k/PFML); tax audit budgeted separately. Confirm payroll is ongoing. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check). Review set to 0:50 per Josephine (CYMA login 5–8 min, complex system; 0.7–1h).</t>
   </si>
   <si>
     <t xml:space="preserve">Newport Classic Cars LLC|1099|1099 Quarterly Review|1099</t>
@@ -4833,11 +4833,11 @@
       </c>
       <c r="F71" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G77*60,0)/1440</f>
-        <v>0.0104166666666667</v>
+        <v>0.0347222222222222</v>
       </c>
       <c r="G71" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G77*Assumptions!$B$5,0)</f>
-        <v>63</v>
+        <v>208</v>
       </c>
       <c r="H71" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L77</f>
@@ -15134,15 +15134,15 @@
         <v>4.6667</v>
       </c>
       <c r="G77" s="15" t="n">
-        <v>0.25</v>
+        <v>0.8333</v>
       </c>
       <c r="H77" s="21" t="n">
         <f aca="false">F77+G77</f>
-        <v>4.9167</v>
+        <v>5.5</v>
       </c>
       <c r="I77" s="2" t="n">
         <f aca="false">ROUND(H77*60,0)</f>
-        <v>295</v>
+        <v>330</v>
       </c>
       <c r="J77" s="2" t="n">
         <f aca="false">ROUND(F77*60,0)</f>
@@ -15150,14 +15150,14 @@
       </c>
       <c r="K77" s="2" t="n">
         <f aca="false">ROUND(G77*60,0)</f>
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="L77" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M77" s="22" t="n">
         <f aca="false">F77*IF(L77="CFO",Assumptions!$B$5,Assumptions!$B$4)+G77*Assumptions!$B$5</f>
-        <v>505.8365</v>
+        <v>651.6615</v>
       </c>
       <c r="N77" s="16" t="n">
         <f aca="false">F77*INDEX(Assumptions!$B$8:$B$14,MATCH(E77,Assumptions!$A$8:$A$14,0))</f>
@@ -15165,7 +15165,7 @@
       </c>
       <c r="O77" s="16" t="n">
         <f aca="false">G77*INDEX(Assumptions!$B$8:$B$14,MATCH(E77,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.25</v>
+        <v>0.8333</v>
       </c>
       <c r="P77" s="28" t="s">
         <v>378</v>
@@ -28919,11 +28919,11 @@
       </c>
       <c r="C34" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A34)</f>
-        <v>1.15285</v>
+        <v>1.73615</v>
       </c>
       <c r="D34" s="35" t="n">
         <f aca="false">B34+C34</f>
-        <v>9.19455</v>
+        <v>9.77785</v>
       </c>
       <c r="E34" s="28" t="s">
         <v>378</v>
@@ -29286,11 +29286,11 @@
       </c>
       <c r="C51" s="19" t="n">
         <f aca="false">SUM(C4:C50)</f>
-        <v>32.4692833333333</v>
+        <v>33.0525833333333</v>
       </c>
       <c r="D51" s="19" t="n">
         <f aca="false">SUM(D4:D50)</f>
-        <v>307.669875</v>
+        <v>308.253175</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -29339,11 +29339,11 @@
       </c>
       <c r="C55" s="4" t="n">
         <f aca="false">C51+C53</f>
-        <v>57.4692833333333</v>
+        <v>58.0525833333333</v>
       </c>
       <c r="D55" s="4" t="n">
         <f aca="false">B55+C55</f>
-        <v>342.669875</v>
+        <v>343.253175</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>

</xml_diff>

<commit_message>
GAV and Young Wealth quarterly review from billing-sheet history (1:30, 1:00)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PRgGtk6aohavQBQTYDwapz
</commit_message>
<xml_diff>
--- a/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
+++ b/budget-hours/Karbon_Budget_Hours_2026-10.xlsx
@@ -1049,7 +1049,7 @@
     <t xml:space="preserve">GAV Enterprises Inc|Accounting|Quarter End Close|Quarterly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</t>
+    <t xml:space="preserve">Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check). Quarterly review from history: Q3 2025 Lisa 1.0 first pass + 0.5 complete = 1.5h; Jan–Jun 2024 review ~1.5h.</t>
   </si>
   <si>
     <t xml:space="preserve">International Alliance Group LLC|1099|1099 Quarterly Review|1099</t>
@@ -1427,7 +1427,7 @@
     <t xml:space="preserve">Young Wealth Management PLLC|Accounting|Quarter End Close|Quarterly</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</t>
+    <t xml:space="preserve">Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check). Quarterly review from history: Lisa Q1–Q2 2025 1.5h (two quarters), Q3 2025 0.7h, Q4 2025 1.25h – about 1h per quarter.</t>
   </si>
   <si>
     <t xml:space="preserve">Work Title</t>
@@ -4337,11 +4337,11 @@
       </c>
       <c r="F55" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G52*60,0)/1440</f>
-        <v>0.0104166666666667</v>
+        <v>0.0625</v>
       </c>
       <c r="G55" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G52*Assumptions!$B$5,0)</f>
-        <v>63</v>
+        <v>375</v>
       </c>
       <c r="H55" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L52</f>
@@ -6290,11 +6290,11 @@
       </c>
       <c r="F118" s="6" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G125*60,0)/1440</f>
-        <v>0.0145833333333333</v>
+        <v>0.0416666666666667</v>
       </c>
       <c r="G118" s="7" t="n">
         <f aca="false">ROUND('Recurring Budgets'!G125*Assumptions!$B$5,0)</f>
-        <v>88</v>
+        <v>250</v>
       </c>
       <c r="H118" s="8" t="str">
         <f aca="false">'Recurring Budgets'!L125</f>
@@ -13814,15 +13814,15 @@
         <v>18.5833</v>
       </c>
       <c r="G52" s="15" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="H52" s="21" t="n">
         <f aca="false">F52+G52</f>
-        <v>18.8333</v>
+        <v>20.0833</v>
       </c>
       <c r="I52" s="2" t="n">
         <f aca="false">ROUND(H52*60,0)</f>
-        <v>1130</v>
+        <v>1205</v>
       </c>
       <c r="J52" s="2" t="n">
         <f aca="false">ROUND(F52*60,0)</f>
@@ -13830,14 +13830,14 @@
       </c>
       <c r="K52" s="2" t="n">
         <f aca="false">ROUND(G52*60,0)</f>
-        <v>15</v>
+        <v>90</v>
       </c>
       <c r="L52" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M52" s="22" t="n">
         <f aca="false">F52*IF(L52="CFO",Assumptions!$B$5,Assumptions!$B$4)+G52*Assumptions!$B$5</f>
-        <v>1827.9135</v>
+        <v>2140.4135</v>
       </c>
       <c r="N52" s="16" t="n">
         <f aca="false">F52*INDEX(Assumptions!$B$8:$B$14,MATCH(E52,Assumptions!$A$8:$A$14,0))</f>
@@ -13845,7 +13845,7 @@
       </c>
       <c r="O52" s="16" t="n">
         <f aca="false">G52*INDEX(Assumptions!$B$8:$B$14,MATCH(E52,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.0833333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="P52" s="25" t="s">
         <v>232</v>
@@ -18166,15 +18166,15 @@
         <v>7.5833</v>
       </c>
       <c r="G125" s="15" t="n">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="H125" s="21" t="n">
         <f aca="false">F125+G125</f>
-        <v>7.9333</v>
+        <v>8.5833</v>
       </c>
       <c r="I125" s="2" t="n">
         <f aca="false">ROUND(H125*60,0)</f>
-        <v>476</v>
+        <v>515</v>
       </c>
       <c r="J125" s="2" t="n">
         <f aca="false">ROUND(F125*60,0)</f>
@@ -18182,14 +18182,14 @@
       </c>
       <c r="K125" s="2" t="n">
         <f aca="false">ROUND(G125*60,0)</f>
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="L125" s="9" t="s">
         <v>87</v>
       </c>
       <c r="M125" s="22" t="n">
         <f aca="false">F125*IF(L125="CFO",Assumptions!$B$5,Assumptions!$B$4)+G125*Assumptions!$B$5</f>
-        <v>807.9135</v>
+        <v>970.4135</v>
       </c>
       <c r="N125" s="16" t="n">
         <f aca="false">F125*INDEX(Assumptions!$B$8:$B$14,MATCH(E125,Assumptions!$A$8:$A$14,0))</f>
@@ -18197,7 +18197,7 @@
       </c>
       <c r="O125" s="16" t="n">
         <f aca="false">G125*INDEX(Assumptions!$B$8:$B$14,MATCH(E125,Assumptions!$A$8:$A$14,0))</f>
-        <v>0.116666666666667</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="P125" s="28" t="s">
         <v>314</v>
@@ -21972,19 +21972,19 @@
       </c>
       <c r="J68" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="K68" s="21" t="n">
         <f aca="false">I68+J68</f>
-        <v>18.8333</v>
+        <v>20.0833</v>
       </c>
       <c r="L68" s="2" t="n">
         <f aca="false">ROUND(K68*60,0)</f>
-        <v>1130</v>
+        <v>1205</v>
       </c>
       <c r="M68" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>1827.9135</v>
+        <v>2140.4135</v>
       </c>
       <c r="N68" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -21992,7 +21992,7 @@
       </c>
       <c r="O68" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P68,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check).</v>
+        <v>Includes Month-end 10.4, Bookkeeping 7.8, CFO advisory 0.7. Review = 0.25h as logged (only 1 reviewed close(s) in Harvest – check). Quarterly review from history: Q3 2025 Lisa 1.0 first pass + 0.5 complete = 1.5h; Jan–Jun 2024 review ~1.5h.</v>
       </c>
       <c r="P68" s="2" t="s">
         <v>337</v>
@@ -28010,19 +28010,19 @@
       </c>
       <c r="J182" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="K182" s="21" t="n">
         <f aca="false">I182+J182</f>
-        <v>7.9333</v>
+        <v>8.5833</v>
       </c>
       <c r="L182" s="2" t="n">
         <f aca="false">ROUND(K182*60,0)</f>
-        <v>476</v>
+        <v>515</v>
       </c>
       <c r="M182" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>807.9135</v>
+        <v>970.4135</v>
       </c>
       <c r="N182" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -28030,7 +28030,7 @@
       </c>
       <c r="O182" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P182,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</v>
+        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check). Quarterly review from history: Lisa Q1–Q2 2025 1.5h (two quarters), Q3 2025 0.7h, Q4 2025 1.25h – about 1h per quarter.</v>
       </c>
       <c r="P182" s="2" t="s">
         <v>463</v>
@@ -28067,19 +28067,19 @@
       </c>
       <c r="J183" s="16" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$G$2:$G$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="K183" s="21" t="n">
         <f aca="false">I183+J183</f>
-        <v>7.9333</v>
+        <v>8.5833</v>
       </c>
       <c r="L183" s="2" t="n">
         <f aca="false">ROUND(K183*60,0)</f>
-        <v>476</v>
+        <v>515</v>
       </c>
       <c r="M183" s="22" t="n">
         <f aca="false">INDEX('Recurring Budgets'!$M$2:$M$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>807.9135</v>
+        <v>970.4135</v>
       </c>
       <c r="N183" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$P$2:$P$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
@@ -28087,7 +28087,7 @@
       </c>
       <c r="O183" s="8" t="str">
         <f aca="false">INDEX('Recurring Budgets'!$Q$2:$Q$125,MATCH(P183,'Recurring Budgets'!$A$2:$A$125,0))</f>
-        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check).</v>
+        <v>Includes Month-end 6.5, Payroll 1.2. Review = 0.35h as logged (only 1 reviewed close(s) in Harvest – check). Quarterly review from history: Lisa Q1–Q2 2025 1.5h (two quarters), Q3 2025 0.7h, Q4 2025 1.25h – about 1h per quarter.</v>
       </c>
       <c r="P183" s="2" t="s">
         <v>463</v>
@@ -28182,19 +28182,19 @@
       </c>
       <c r="J186" s="4" t="n">
         <f aca="false">SUM(J2:J184)</f>
-        <v>51.8331</v>
+        <v>54.3831</v>
       </c>
       <c r="K186" s="4" t="n">
         <f aca="false">SUM(K2:K184)</f>
-        <v>602.5624</v>
+        <v>605.1124</v>
       </c>
       <c r="L186" s="4" t="n">
         <f aca="false">SUM(L2:L184)</f>
-        <v>36158</v>
+        <v>36311</v>
       </c>
       <c r="M186" s="32" t="n">
         <f aca="false">SUM(M2:M184)</f>
-        <v>72381.7355</v>
+        <v>73019.2355</v>
       </c>
       <c r="N186" s="2"/>
       <c r="O186" s="2"/>
@@ -28768,11 +28768,11 @@
       </c>
       <c r="C27" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A27)</f>
-        <v>0.0833333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="D27" s="35" t="n">
         <f aca="false">B27+C27</f>
-        <v>6.58331666666667</v>
+        <v>6.99998333333333</v>
       </c>
       <c r="E27" s="25" t="s">
         <v>232</v>
@@ -29265,11 +29265,11 @@
       </c>
       <c r="C50" s="34" t="n">
         <f aca="false">SUMIFS('Recurring Budgets'!$O$2:$O$125,'Recurring Budgets'!$B$2:$B$125,A50)</f>
-        <v>0.116666666666667</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="D50" s="35" t="n">
         <f aca="false">B50+C50</f>
-        <v>2.89443333333333</v>
+        <v>3.1111</v>
       </c>
       <c r="E50" s="28" t="s">
         <v>314</v>
@@ -29286,11 +29286,11 @@
       </c>
       <c r="C51" s="19" t="n">
         <f aca="false">SUM(C4:C50)</f>
-        <v>33.0525833333333</v>
+        <v>33.6859166666667</v>
       </c>
       <c r="D51" s="19" t="n">
         <f aca="false">SUM(D4:D50)</f>
-        <v>308.253175</v>
+        <v>308.886508333333</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -29339,11 +29339,11 @@
       </c>
       <c r="C55" s="4" t="n">
         <f aca="false">C51+C53</f>
-        <v>58.0525833333333</v>
+        <v>58.6859166666667</v>
       </c>
       <c r="D55" s="4" t="n">
         <f aca="false">B55+C55</f>
-        <v>343.253175</v>
+        <v>343.886508333333</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>

</xml_diff>